<commit_message>
Commit from GitHub Actions (Go)
</commit_message>
<xml_diff>
--- a/raw/uncategorized/311 Windsor Contact Centre Metrics 2025.xlsx
+++ b/raw/uncategorized/311 Windsor Contact Centre Metrics 2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Administration\Reports\Open Data Call Centre Metrics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1932B6CC-D9DD-4C1B-920E-59D8D7B6C2A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{735E7ABA-7485-474D-8771-800DED8B543D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="750" yWindow="2175" windowWidth="14400" windowHeight="10665" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2016 - 2024" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
         <v>5</v>
       </c>
       <c r="B3" s="24">
-        <v>114941</v>
+        <v>115628</v>
       </c>
       <c r="C3" s="8">
         <v>102591</v>

</xml_diff>